<commit_message>
All is working and and just need to align the coulmes needed, thats all
</commit_message>
<xml_diff>
--- a/restructured_parten.xlsx
+++ b/restructured_parten.xlsx
@@ -34,94 +34,94 @@
     <t>Plant</t>
   </si>
   <si>
+    <t>A/T(TRB)+,CMB(BZ)+</t>
+  </si>
+  <si>
+    <t>CMB(GA)+,PC(C513)-</t>
+  </si>
+  <si>
+    <t>CC(1.3)+,CMB(GA)+,ECO(PL8)+,PC(C513)+</t>
+  </si>
+  <si>
+    <t>CC(2.2)+</t>
+  </si>
+  <si>
+    <t>MY(26)+</t>
+  </si>
+  <si>
     <t>CC(2.2)+,CMB(DS)+</t>
   </si>
   <si>
-    <t>CC(2.2)+</t>
-  </si>
-  <si>
-    <t>A/T(TRB)+,CMB(BZ)+</t>
+    <t>CMB(DS)-,TT(4X4)+</t>
+  </si>
+  <si>
+    <t>AM(11)+</t>
   </si>
   <si>
     <t>CMB(GA)+,MY(26)+,PC(CA79)+</t>
   </si>
   <si>
-    <t>CMB(DS)-,TT(4X4)+</t>
-  </si>
-  <si>
-    <t>CMB(GA)+,PC(C513)-</t>
-  </si>
-  <si>
-    <t>AM(11)+</t>
-  </si>
-  <si>
-    <t>CC(1.3)+,CMB(GA)+,ECO(PL8)+,PC(C513)+</t>
-  </si>
-  <si>
-    <t>MY(26)+</t>
+    <t>029,392</t>
+  </si>
+  <si>
+    <t>029,097,392</t>
   </si>
   <si>
     <t>RDG</t>
   </si>
   <si>
-    <t>029,392</t>
-  </si>
-  <si>
-    <t>029,097,392</t>
-  </si>
-  <si>
     <t>097</t>
   </si>
   <si>
+    <t>MY(26)+,097-,(029,392)+</t>
+  </si>
+  <si>
+    <t>MY(26)+,(029,097,392)+</t>
+  </si>
+  <si>
+    <t>AM(11)+,RDG+</t>
+  </si>
+  <si>
     <t>CMB(GA)+,MY(26)+,PC(CA79)+,</t>
   </si>
   <si>
-    <t>AM(11)+,RDG+</t>
-  </si>
-  <si>
-    <t>MY(26)+,097-,(029,392)+</t>
-  </si>
-  <si>
-    <t>MY(26)+,(029,097,392)+</t>
+    <t>265</t>
   </si>
   <si>
     <t>551</t>
   </si>
   <si>
+    <t>376</t>
+  </si>
+  <si>
+    <t>291</t>
+  </si>
+  <si>
+    <t>598</t>
+  </si>
+  <si>
+    <t>358</t>
+  </si>
+  <si>
+    <t>281</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>363</t>
+  </si>
+  <si>
+    <t>341</t>
+  </si>
+  <si>
     <t>226</t>
   </si>
   <si>
-    <t>376</t>
-  </si>
-  <si>
-    <t>265</t>
-  </si>
-  <si>
-    <t>358</t>
-  </si>
-  <si>
-    <t>281</t>
-  </si>
-  <si>
-    <t>341</t>
-  </si>
-  <si>
-    <t>363</t>
-  </si>
-  <si>
-    <t>521</t>
-  </si>
-  <si>
-    <t>598</t>
-  </si>
-  <si>
-    <t>291</t>
+    <t>FIASA</t>
   </si>
   <si>
     <t>FIAPE</t>
-  </si>
-  <si>
-    <t>FIASA</t>
   </si>
 </sst>
 </file>
@@ -527,7 +527,7 @@
         <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -541,7 +541,7 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -583,7 +583,7 @@
         <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -597,7 +597,7 @@
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -653,7 +653,7 @@
         <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -681,7 +681,7 @@
         <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -695,7 +695,7 @@
         <v>25</v>
       </c>
       <c r="F15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -737,7 +737,7 @@
         <v>28</v>
       </c>
       <c r="F18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -751,7 +751,7 @@
         <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -807,7 +807,7 @@
         <v>33</v>
       </c>
       <c r="F23" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -835,7 +835,7 @@
         <v>24</v>
       </c>
       <c r="F25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -849,7 +849,7 @@
         <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -891,7 +891,7 @@
         <v>28</v>
       </c>
       <c r="F29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -905,7 +905,7 @@
         <v>29</v>
       </c>
       <c r="F30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -961,7 +961,7 @@
         <v>33</v>
       </c>
       <c r="F34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -969,7 +969,7 @@
         <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E35" t="s">
         <v>23</v>
@@ -983,13 +983,13 @@
         <v>9</v>
       </c>
       <c r="D36" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E36" t="s">
         <v>24</v>
       </c>
       <c r="F36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -997,13 +997,13 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E37" t="s">
         <v>25</v>
       </c>
       <c r="F37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1011,7 +1011,7 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E38" t="s">
         <v>26</v>
@@ -1025,7 +1025,7 @@
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E39" t="s">
         <v>27</v>
@@ -1039,13 +1039,13 @@
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E40" t="s">
         <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1053,13 +1053,13 @@
         <v>9</v>
       </c>
       <c r="D41" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E41" t="s">
         <v>29</v>
       </c>
       <c r="F41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1067,7 +1067,7 @@
         <v>9</v>
       </c>
       <c r="D42" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E42" t="s">
         <v>30</v>
@@ -1081,7 +1081,7 @@
         <v>9</v>
       </c>
       <c r="D43" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E43" t="s">
         <v>31</v>
@@ -1095,7 +1095,7 @@
         <v>9</v>
       </c>
       <c r="D44" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E44" t="s">
         <v>32</v>
@@ -1109,21 +1109,27 @@
         <v>9</v>
       </c>
       <c r="D45" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E45" t="s">
         <v>33</v>
       </c>
       <c r="F45" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>10</v>
       </c>
+      <c r="B46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
       <c r="D46" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E46" t="s">
         <v>23</v>
@@ -1136,36 +1142,54 @@
       <c r="A47" t="s">
         <v>10</v>
       </c>
+      <c r="B47" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
       <c r="D47" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E47" t="s">
         <v>24</v>
       </c>
       <c r="F47" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>10</v>
       </c>
+      <c r="B48" t="s">
+        <v>15</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
       <c r="D48" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E48" t="s">
         <v>25</v>
       </c>
       <c r="F48" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>10</v>
       </c>
+      <c r="B49" t="s">
+        <v>15</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
       <c r="D49" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E49" t="s">
         <v>26</v>
@@ -1178,8 +1202,14 @@
       <c r="A50" t="s">
         <v>10</v>
       </c>
+      <c r="B50" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" t="s">
+        <v>18</v>
+      </c>
       <c r="D50" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E50" t="s">
         <v>27</v>
@@ -1192,36 +1222,54 @@
       <c r="A51" t="s">
         <v>10</v>
       </c>
+      <c r="B51" t="s">
+        <v>15</v>
+      </c>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
       <c r="D51" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E51" t="s">
         <v>28</v>
       </c>
       <c r="F51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>10</v>
       </c>
+      <c r="B52" t="s">
+        <v>15</v>
+      </c>
+      <c r="C52" t="s">
+        <v>18</v>
+      </c>
       <c r="D52" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E52" t="s">
         <v>29</v>
       </c>
       <c r="F52" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>10</v>
       </c>
+      <c r="B53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C53" t="s">
+        <v>18</v>
+      </c>
       <c r="D53" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E53" t="s">
         <v>30</v>
@@ -1234,8 +1282,14 @@
       <c r="A54" t="s">
         <v>10</v>
       </c>
+      <c r="B54" t="s">
+        <v>15</v>
+      </c>
+      <c r="C54" t="s">
+        <v>18</v>
+      </c>
       <c r="D54" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E54" t="s">
         <v>31</v>
@@ -1248,8 +1302,14 @@
       <c r="A55" t="s">
         <v>10</v>
       </c>
+      <c r="B55" t="s">
+        <v>15</v>
+      </c>
+      <c r="C55" t="s">
+        <v>18</v>
+      </c>
       <c r="D55" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E55" t="s">
         <v>32</v>
@@ -1262,22 +1322,31 @@
       <c r="A56" t="s">
         <v>10</v>
       </c>
+      <c r="B56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" t="s">
+        <v>18</v>
+      </c>
       <c r="D56" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E56" t="s">
         <v>33</v>
       </c>
       <c r="F56" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B57" t="s">
+        <v>16</v>
       </c>
       <c r="D57" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E57" t="s">
         <v>23</v>
@@ -1288,38 +1357,47 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B58" t="s">
+        <v>16</v>
       </c>
       <c r="D58" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E58" t="s">
         <v>24</v>
       </c>
       <c r="F58" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B59" t="s">
+        <v>16</v>
       </c>
       <c r="D59" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E59" t="s">
         <v>25</v>
       </c>
       <c r="F59" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B60" t="s">
+        <v>16</v>
       </c>
       <c r="D60" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E60" t="s">
         <v>26</v>
@@ -1330,10 +1408,13 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
+        <v>16</v>
       </c>
       <c r="D61" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E61" t="s">
         <v>27</v>
@@ -1344,38 +1425,47 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B62" t="s">
+        <v>16</v>
       </c>
       <c r="D62" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E62" t="s">
         <v>28</v>
       </c>
       <c r="F62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B63" t="s">
+        <v>16</v>
       </c>
       <c r="D63" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E63" t="s">
         <v>29</v>
       </c>
       <c r="F63" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B64" t="s">
+        <v>16</v>
       </c>
       <c r="D64" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E64" t="s">
         <v>30</v>
@@ -1386,10 +1476,13 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B65" t="s">
+        <v>16</v>
       </c>
       <c r="D65" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E65" t="s">
         <v>31</v>
@@ -1400,10 +1493,13 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B66" t="s">
+        <v>16</v>
       </c>
       <c r="D66" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E66" t="s">
         <v>32</v>
@@ -1414,27 +1510,27 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="B67" t="s">
+        <v>16</v>
       </c>
       <c r="D67" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E67" t="s">
         <v>33</v>
       </c>
       <c r="F67" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>12</v>
-      </c>
-      <c r="B68" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D68" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E68" t="s">
         <v>23</v>
@@ -1445,47 +1541,38 @@
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>12</v>
-      </c>
-      <c r="B69" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D69" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E69" t="s">
         <v>24</v>
       </c>
       <c r="F69" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" t="s">
-        <v>12</v>
-      </c>
-      <c r="B70" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D70" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E70" t="s">
         <v>25</v>
       </c>
       <c r="F70" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" t="s">
-        <v>12</v>
-      </c>
-      <c r="B71" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D71" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E71" t="s">
         <v>26</v>
@@ -1496,13 +1583,10 @@
     </row>
     <row r="72" spans="1:6">
       <c r="A72" t="s">
-        <v>12</v>
-      </c>
-      <c r="B72" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D72" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E72" t="s">
         <v>27</v>
@@ -1513,47 +1597,38 @@
     </row>
     <row r="73" spans="1:6">
       <c r="A73" t="s">
-        <v>12</v>
-      </c>
-      <c r="B73" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D73" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E73" t="s">
         <v>28</v>
       </c>
       <c r="F73" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="74" spans="1:6">
       <c r="A74" t="s">
-        <v>12</v>
-      </c>
-      <c r="B74" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D74" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E74" t="s">
         <v>29</v>
       </c>
       <c r="F74" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" t="s">
-        <v>12</v>
-      </c>
-      <c r="B75" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D75" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E75" t="s">
         <v>30</v>
@@ -1564,13 +1639,10 @@
     </row>
     <row r="76" spans="1:6">
       <c r="A76" t="s">
-        <v>12</v>
-      </c>
-      <c r="B76" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D76" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E76" t="s">
         <v>31</v>
@@ -1581,13 +1653,10 @@
     </row>
     <row r="77" spans="1:6">
       <c r="A77" t="s">
-        <v>12</v>
-      </c>
-      <c r="B77" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D77" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E77" t="s">
         <v>32</v>
@@ -1598,27 +1667,24 @@
     </row>
     <row r="78" spans="1:6">
       <c r="A78" t="s">
-        <v>12</v>
-      </c>
-      <c r="B78" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D78" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E78" t="s">
         <v>33</v>
       </c>
       <c r="F78" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E79" t="s">
         <v>23</v>
@@ -1629,38 +1695,38 @@
     </row>
     <row r="80" spans="1:6">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D80" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E80" t="s">
         <v>24</v>
       </c>
       <c r="F80" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E81" t="s">
         <v>25</v>
       </c>
       <c r="F81" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E82" t="s">
         <v>26</v>
@@ -1671,10 +1737,10 @@
     </row>
     <row r="83" spans="1:6">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E83" t="s">
         <v>27</v>
@@ -1685,38 +1751,38 @@
     </row>
     <row r="84" spans="1:6">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D84" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E84" t="s">
         <v>28</v>
       </c>
       <c r="F84" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D85" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E85" t="s">
         <v>29</v>
       </c>
       <c r="F85" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E86" t="s">
         <v>30</v>
@@ -1727,10 +1793,10 @@
     </row>
     <row r="87" spans="1:6">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D87" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E87" t="s">
         <v>31</v>
@@ -1741,10 +1807,10 @@
     </row>
     <row r="88" spans="1:6">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D88" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E88" t="s">
         <v>32</v>
@@ -1755,27 +1821,24 @@
     </row>
     <row r="89" spans="1:6">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E89" t="s">
         <v>33</v>
       </c>
       <c r="F89" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>16</v>
-      </c>
-      <c r="C90" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D90" t="s">
         <v>21</v>
@@ -1789,13 +1852,10 @@
     </row>
     <row r="91" spans="1:6">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
-        <v>16</v>
-      </c>
-      <c r="C91" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D91" t="s">
         <v>21</v>
@@ -1804,18 +1864,15 @@
         <v>24</v>
       </c>
       <c r="F91" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>16</v>
-      </c>
-      <c r="C92" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D92" t="s">
         <v>21</v>
@@ -1824,18 +1881,15 @@
         <v>25</v>
       </c>
       <c r="F92" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>16</v>
-      </c>
-      <c r="C93" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D93" t="s">
         <v>21</v>
@@ -1849,13 +1903,10 @@
     </row>
     <row r="94" spans="1:6">
       <c r="A94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>16</v>
-      </c>
-      <c r="C94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D94" t="s">
         <v>21</v>
@@ -1869,13 +1920,10 @@
     </row>
     <row r="95" spans="1:6">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>16</v>
-      </c>
-      <c r="C95" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D95" t="s">
         <v>21</v>
@@ -1884,18 +1932,15 @@
         <v>28</v>
       </c>
       <c r="F95" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>16</v>
-      </c>
-      <c r="C96" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D96" t="s">
         <v>21</v>
@@ -1904,18 +1949,15 @@
         <v>29</v>
       </c>
       <c r="F96" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B97" t="s">
-        <v>16</v>
-      </c>
-      <c r="C97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D97" t="s">
         <v>21</v>
@@ -1929,13 +1971,10 @@
     </row>
     <row r="98" spans="1:6">
       <c r="A98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
-        <v>16</v>
-      </c>
-      <c r="C98" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D98" t="s">
         <v>21</v>
@@ -1949,13 +1988,10 @@
     </row>
     <row r="99" spans="1:6">
       <c r="A99" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
-        <v>16</v>
-      </c>
-      <c r="C99" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D99" t="s">
         <v>21</v>
@@ -1969,13 +2005,10 @@
     </row>
     <row r="100" spans="1:6">
       <c r="A100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B100" t="s">
-        <v>16</v>
-      </c>
-      <c r="C100" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D100" t="s">
         <v>21</v>
@@ -1984,16 +2017,13 @@
         <v>33</v>
       </c>
       <c r="F100" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" t="s">
         <v>14</v>
       </c>
-      <c r="B101" t="s">
-        <v>17</v>
-      </c>
       <c r="D101" t="s">
         <v>22</v>
       </c>
@@ -2008,9 +2038,6 @@
       <c r="A102" t="s">
         <v>14</v>
       </c>
-      <c r="B102" t="s">
-        <v>17</v>
-      </c>
       <c r="D102" t="s">
         <v>22</v>
       </c>
@@ -2018,16 +2045,13 @@
         <v>24</v>
       </c>
       <c r="F102" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" t="s">
         <v>14</v>
       </c>
-      <c r="B103" t="s">
-        <v>17</v>
-      </c>
       <c r="D103" t="s">
         <v>22</v>
       </c>
@@ -2035,16 +2059,13 @@
         <v>25</v>
       </c>
       <c r="F103" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104" spans="1:6">
       <c r="A104" t="s">
         <v>14</v>
       </c>
-      <c r="B104" t="s">
-        <v>17</v>
-      </c>
       <c r="D104" t="s">
         <v>22</v>
       </c>
@@ -2059,9 +2080,6 @@
       <c r="A105" t="s">
         <v>14</v>
       </c>
-      <c r="B105" t="s">
-        <v>17</v>
-      </c>
       <c r="D105" t="s">
         <v>22</v>
       </c>
@@ -2076,9 +2094,6 @@
       <c r="A106" t="s">
         <v>14</v>
       </c>
-      <c r="B106" t="s">
-        <v>17</v>
-      </c>
       <c r="D106" t="s">
         <v>22</v>
       </c>
@@ -2086,16 +2101,13 @@
         <v>28</v>
       </c>
       <c r="F106" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" t="s">
         <v>14</v>
       </c>
-      <c r="B107" t="s">
-        <v>17</v>
-      </c>
       <c r="D107" t="s">
         <v>22</v>
       </c>
@@ -2103,16 +2115,13 @@
         <v>29</v>
       </c>
       <c r="F107" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" t="s">
         <v>14</v>
       </c>
-      <c r="B108" t="s">
-        <v>17</v>
-      </c>
       <c r="D108" t="s">
         <v>22</v>
       </c>
@@ -2127,9 +2136,6 @@
       <c r="A109" t="s">
         <v>14</v>
       </c>
-      <c r="B109" t="s">
-        <v>17</v>
-      </c>
       <c r="D109" t="s">
         <v>22</v>
       </c>
@@ -2144,9 +2150,6 @@
       <c r="A110" t="s">
         <v>14</v>
       </c>
-      <c r="B110" t="s">
-        <v>17</v>
-      </c>
       <c r="D110" t="s">
         <v>22</v>
       </c>
@@ -2161,9 +2164,6 @@
       <c r="A111" t="s">
         <v>14</v>
       </c>
-      <c r="B111" t="s">
-        <v>17</v>
-      </c>
       <c r="D111" t="s">
         <v>22</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>33</v>
       </c>
       <c r="F111" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>